<commit_message>
final change 1 with MDL and TP
</commit_message>
<xml_diff>
--- a/uploaded_royalty.xlsx
+++ b/uploaded_royalty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kpras\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB0585D-9D00-4FF6-B6B4-847A55E686B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF17181F-E32C-49D7-992C-9DF9635C8D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31065" yWindow="2265" windowWidth="21600" windowHeight="11235" xr2:uid="{3423368E-0AEA-42EB-973E-FF4BDDAFC8B8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3423368E-0AEA-42EB-973E-FF4BDDAFC8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="35">
   <si>
     <t>AP31TN5227</t>
   </si>
@@ -87,22 +87,49 @@
     <t>Dispatch Quantity</t>
   </si>
   <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>M Sand</t>
-  </si>
-  <si>
-    <t>TMGA17438845</t>
-  </si>
-  <si>
-    <t>TMGA17438939</t>
-  </si>
-  <si>
-    <t>TMGA17439122</t>
-  </si>
-  <si>
-    <t>TMGA17439971</t>
+    <t>20MM</t>
+  </si>
+  <si>
+    <t>10MM</t>
+  </si>
+  <si>
+    <t>MDL ID</t>
+  </si>
+  <si>
+    <t>M302024216</t>
+  </si>
+  <si>
+    <t>TMGA29779818</t>
+  </si>
+  <si>
+    <t>TMGA29779819</t>
+  </si>
+  <si>
+    <t>TMGA29779820</t>
+  </si>
+  <si>
+    <t>TMGA29779821</t>
+  </si>
+  <si>
+    <t>TMGA29779822</t>
+  </si>
+  <si>
+    <t>TMGA29779823</t>
+  </si>
+  <si>
+    <t>TMGA29779824</t>
+  </si>
+  <si>
+    <t>TMGA29779825</t>
+  </si>
+  <si>
+    <t>TMGA29779826</t>
+  </si>
+  <si>
+    <t>TMGA29779827</t>
+  </si>
+  <si>
+    <t>TMGA29779828</t>
   </si>
 </sst>
 </file>
@@ -145,7 +172,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -168,52 +195,25 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,20 +528,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71C02794-A52F-486F-A82D-7D101F9BFE71}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -552,141 +551,354 @@
         <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>14</v>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="4">
-        <v>9908076542</v>
-      </c>
-      <c r="D2" s="5">
-        <v>40</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="4">
-        <v>9908076542</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="6">
-        <v>5500</v>
+      <c r="C2" s="2">
+        <v>9121723275</v>
+      </c>
+      <c r="D2" s="2">
+        <v>40</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="2">
+        <v>9908076542</v>
+      </c>
+      <c r="D3" s="2">
+        <v>40</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2">
         <v>8374066219</v>
       </c>
-      <c r="D3" s="5">
-        <v>40</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="D4" s="2">
+        <v>40</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="2">
+        <v>9959035842</v>
+      </c>
+      <c r="D5" s="2">
+        <v>40</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="2">
+        <v>9121723275</v>
+      </c>
+      <c r="D6" s="2">
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2">
+        <v>9908076542</v>
+      </c>
+      <c r="D7" s="2">
+        <v>40</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2">
         <v>8374066219</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="D8" s="2">
+        <v>40</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="6">
-        <v>5500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="H8" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2">
+        <v>9959035842</v>
+      </c>
+      <c r="D9" s="2">
+        <v>40</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="2">
+        <v>9121723275</v>
+      </c>
+      <c r="D10" s="2">
+        <v>40</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="2">
+        <v>9908076542</v>
+      </c>
+      <c r="D11" s="2">
+        <v>40</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4">
-        <v>9959035842</v>
-      </c>
-      <c r="D4" s="5">
-        <v>40</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="4">
-        <v>9959035842</v>
-      </c>
-      <c r="H4" s="4" t="s">
+      <c r="B12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="2">
+        <v>8374066219</v>
+      </c>
+      <c r="D12" s="2">
+        <v>40</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="6">
-        <v>5500</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="H12" s="3">
+        <v>5500</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4">
-        <v>9121723275</v>
-      </c>
-      <c r="D5" s="5">
-        <v>40</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G5" s="4">
-        <v>9121723275</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="6">
-        <v>5500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>